<commit_message>
Comparativa de descripción vs transcripción
</commit_message>
<xml_diff>
--- a/podcast-data/Punzadas_Sonoras_referencias.xlsx
+++ b/podcast-data/Punzadas_Sonoras_referencias.xlsx
@@ -13164,21 +13164,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O158" s="2" t="inlineStr">
-        <is>
-          <t>Fancy Ediciones</t>
-        </is>
-      </c>
-      <c r="P158" s="2" t="inlineStr">
-        <is>
-          <t>2007</t>
-        </is>
-      </c>
-      <c r="Q158" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O158" s="2" t="inlineStr"/>
+      <c r="P158" s="2" t="inlineStr"/>
+      <c r="Q158" s="2" t="inlineStr"/>
       <c r="R158" s="2" t="inlineStr">
         <is>
           <t>no — título normalizado o inferido</t>
@@ -25421,7 +25409,7 @@
       </c>
       <c r="P308" s="2" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="Q308" s="2" t="inlineStr">
@@ -25860,21 +25848,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O313" s="2" t="inlineStr">
-        <is>
-          <t>Aguado Rubira, Pedro Francisco</t>
-        </is>
-      </c>
-      <c r="P313" s="2" t="inlineStr">
-        <is>
-          <t>2008</t>
-        </is>
-      </c>
-      <c r="Q313" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O313" s="2" t="inlineStr"/>
+      <c r="P313" s="2" t="inlineStr"/>
+      <c r="Q313" s="2" t="inlineStr"/>
       <c r="R313" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -30087,7 +30063,7 @@
       </c>
       <c r="P364" s="2" t="inlineStr">
         <is>
-          <t>1886</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="Q364" s="2" t="inlineStr">
@@ -30363,7 +30339,7 @@
       </c>
       <c r="P367" s="2" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="Q367" s="2" t="inlineStr">
@@ -31374,21 +31350,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O379" s="2" t="inlineStr">
-        <is>
-          <t>Editorial Verbum, S.L.</t>
-        </is>
-      </c>
-      <c r="P379" s="2" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
-      <c r="Q379" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O379" s="2" t="inlineStr"/>
+      <c r="P379" s="2" t="inlineStr"/>
+      <c r="Q379" s="2" t="inlineStr"/>
       <c r="R379" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -33720,21 +33684,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O406" s="2" t="inlineStr">
-        <is>
-          <t>Sar Alejandria Ediciones</t>
-        </is>
-      </c>
-      <c r="P406" s="2" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="Q406" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O406" s="2" t="inlineStr"/>
+      <c r="P406" s="2" t="inlineStr"/>
+      <c r="Q406" s="2" t="inlineStr"/>
       <c r="R406" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -35816,21 +35768,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O431" s="2" t="inlineStr">
-        <is>
-          <t>Harlequin Ibérica</t>
-        </is>
-      </c>
-      <c r="P431" s="2" t="inlineStr">
-        <is>
-          <t>1991</t>
-        </is>
-      </c>
-      <c r="Q431" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O431" s="2" t="inlineStr"/>
+      <c r="P431" s="2" t="inlineStr"/>
+      <c r="Q431" s="2" t="inlineStr"/>
       <c r="R431" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -36677,7 +36617,7 @@
       </c>
       <c r="P441" s="2" t="inlineStr">
         <is>
-          <t>2097</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="Q441" s="2" t="inlineStr">
@@ -36939,7 +36879,7 @@
       </c>
       <c r="P444" s="2" t="inlineStr">
         <is>
-          <t>1989</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="Q444" s="2" t="inlineStr">
@@ -37111,7 +37051,7 @@
       </c>
       <c r="P446" s="2" t="inlineStr">
         <is>
-          <t>1885</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="Q446" s="2" t="inlineStr">
@@ -38387,7 +38327,7 @@
       </c>
       <c r="P461" s="2" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="Q461" s="2" t="inlineStr">
@@ -39243,7 +39183,7 @@
       </c>
       <c r="P471" s="2" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="Q471" s="2" t="inlineStr">
@@ -39852,21 +39792,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O478" s="2" t="inlineStr">
-        <is>
-          <t>Axóuxere Editora</t>
-        </is>
-      </c>
-      <c r="P478" s="2" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="Q478" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O478" s="2" t="inlineStr"/>
+      <c r="P478" s="2" t="inlineStr"/>
+      <c r="Q478" s="2" t="inlineStr"/>
       <c r="R478" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -40628,21 +40556,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O487" s="2" t="inlineStr">
-        <is>
-          <t>Nova Terra, S.A.</t>
-        </is>
-      </c>
-      <c r="P487" s="2" t="inlineStr">
-        <is>
-          <t>1969</t>
-        </is>
-      </c>
-      <c r="Q487" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O487" s="2" t="inlineStr"/>
+      <c r="P487" s="2" t="inlineStr"/>
+      <c r="Q487" s="2" t="inlineStr"/>
       <c r="R487" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -41068,21 +40984,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O492" s="2" t="inlineStr">
-        <is>
-          <t>Babidi-Bú</t>
-        </is>
-      </c>
-      <c r="P492" s="2" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="Q492" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O492" s="2" t="inlineStr"/>
+      <c r="P492" s="2" t="inlineStr"/>
+      <c r="Q492" s="2" t="inlineStr"/>
       <c r="R492" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -41368,7 +41272,7 @@
       </c>
       <c r="Q495" s="2" t="inlineStr">
         <is>
-          <t>MCU — inferido</t>
+          <t>MCU — verificado</t>
         </is>
       </c>
       <c r="R495" s="2" t="inlineStr">
@@ -42140,7 +42044,7 @@
       </c>
       <c r="Q504" s="2" t="inlineStr">
         <is>
-          <t>MCU — inferido</t>
+          <t>MCU — verificado</t>
         </is>
       </c>
       <c r="R504" s="2" t="inlineStr">
@@ -43420,21 +43324,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O519" s="2" t="inlineStr">
-        <is>
-          <t>Instituto de Estadística y Cartografía de Andalucía</t>
-        </is>
-      </c>
-      <c r="P519" s="2" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
-      </c>
-      <c r="Q519" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O519" s="2" t="inlineStr"/>
+      <c r="P519" s="2" t="inlineStr"/>
+      <c r="Q519" s="2" t="inlineStr"/>
       <c r="R519" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -44069,7 +43961,7 @@
       </c>
       <c r="P526" s="2" t="inlineStr">
         <is>
-          <t>1925</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="Q526" s="2" t="inlineStr">
@@ -46244,21 +46136,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O551" s="2" t="inlineStr">
-        <is>
-          <t>Abenójar Sanjuán, Óscar</t>
-        </is>
-      </c>
-      <c r="P551" s="2" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="Q551" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O551" s="2" t="inlineStr"/>
+      <c r="P551" s="2" t="inlineStr"/>
+      <c r="Q551" s="2" t="inlineStr"/>
       <c r="R551" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -49384,7 +49264,7 @@
       </c>
       <c r="Q587" s="2" t="inlineStr">
         <is>
-          <t>MCU — inferido</t>
+          <t>MCU — verificado</t>
         </is>
       </c>
       <c r="R587" s="2" t="inlineStr">
@@ -50360,7 +50240,7 @@
       </c>
       <c r="Q598" s="2" t="inlineStr">
         <is>
-          <t>MCU — inferido</t>
+          <t>MCU — verificado</t>
         </is>
       </c>
       <c r="R598" s="2" t="inlineStr">
@@ -50451,7 +50331,7 @@
       </c>
       <c r="P599" s="2" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="Q599" s="2" t="inlineStr">
@@ -52634,21 +52514,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O624" s="2" t="inlineStr">
-        <is>
-          <t>Badenes Bou, María Elena</t>
-        </is>
-      </c>
-      <c r="P624" s="2" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="Q624" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O624" s="2" t="inlineStr"/>
+      <c r="P624" s="2" t="inlineStr"/>
+      <c r="Q624" s="2" t="inlineStr"/>
       <c r="R624" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -53619,7 +53487,7 @@
       </c>
       <c r="P636" s="2" t="inlineStr">
         <is>
-          <t>2007</t>
+          <t>2004</t>
         </is>
       </c>
       <c r="Q636" s="2" t="inlineStr">
@@ -53702,21 +53570,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O637" s="2" t="inlineStr">
-        <is>
-          <t>Ediciones Encuentro, S.A.</t>
-        </is>
-      </c>
-      <c r="P637" s="2" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="Q637" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O637" s="2" t="inlineStr"/>
+      <c r="P637" s="2" t="inlineStr"/>
+      <c r="Q637" s="2" t="inlineStr"/>
       <c r="R637" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -56416,21 +56272,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O669" s="2" t="inlineStr">
-        <is>
-          <t>De Vecchi Ediciones, S.A.</t>
-        </is>
-      </c>
-      <c r="P669" s="2" t="inlineStr">
-        <is>
-          <t>1996</t>
-        </is>
-      </c>
-      <c r="Q669" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O669" s="2" t="inlineStr"/>
+      <c r="P669" s="2" t="inlineStr"/>
+      <c r="Q669" s="2" t="inlineStr"/>
       <c r="R669" s="2" t="inlineStr">
         <is>
           <t>sí</t>
@@ -56598,21 +56442,9 @@
           <t>sin datos</t>
         </is>
       </c>
-      <c r="O671" s="2" t="inlineStr">
-        <is>
-          <t>Álvarez Álvarez, Covadonga</t>
-        </is>
-      </c>
-      <c r="P671" s="2" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="Q671" s="2" t="inlineStr">
-        <is>
-          <t>MCU — inferido</t>
-        </is>
-      </c>
+      <c r="O671" s="2" t="inlineStr"/>
+      <c r="P671" s="2" t="inlineStr"/>
+      <c r="Q671" s="2" t="inlineStr"/>
       <c r="R671" s="2" t="inlineStr">
         <is>
           <t>sí</t>

</xml_diff>